<commit_message>
Audit robot arm workbooks against SO-101 and LeKiwi docs
</commit_message>
<xml_diff>
--- a/Robot Arm Parts - Highest.xlsx
+++ b/Robot Arm Parts - Highest.xlsx
@@ -398,21 +398,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H35"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="80.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Highest</v>
       </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -421,6 +432,50 @@
       <c r="B2" t="str">
         <v>2026-02-28</v>
       </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -499,7 +554,7 @@
         <v>20.4</v>
       </c>
       <c r="H6" t="str">
-        <v>Exact ST/SC serial bus board for the leader arm.</v>
+        <v>Exact repo board ASIN. LeRobot requires ST/SC serial bus support and B-channel jumpers during setup. Official board docs list 9-12.6V input, which conflicts with the repo's 5V leader PSU guidance.</v>
       </c>
     </row>
     <row r="7">
@@ -534,26 +589,26 @@
         <v>Leader</v>
       </c>
       <c r="B8" t="str">
-        <v>5V 5A Power Adapter 25W AC 100-240V to DC Wall Power Supply Converter with 5.5x2.5mm/2.1mm Plug</v>
+        <v>Facmogu DC 5V 4A AC to DC Converter, AC 100-240V to DC 5 Volt 4 Amp 20W Power Supply 5V Switching Transformer Power Adapter, Wall Mounted Adapter with with Barrel Connector 5.5x2.5mm &amp; 5.5x2.1mm</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="str">
-        <v>https://www.amazon.ca/MTDZKJG-100-240V-Converter-5-5x2-5mm-Security/dp/B0CJHQNFMG</v>
+        <v>https://www.amazon.ca/Facmogu-Switching-Transformer-Converter-Compatible/dp/B087LY41PV</v>
       </c>
       <c r="E8">
-        <v>26.41</v>
+        <v>14.39</v>
       </c>
       <c r="F8">
-        <v>5.51</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <f>C8*E8+F8</f>
-        <v>31.92</v>
+        <v>14.39</v>
       </c>
       <c r="H8" t="str">
-        <v>Leader-side power supply with 5.5x2.1mm compatibility.</v>
+        <v>Exact SO-101 repo PSU ASIN. Upstream controller-board voltage guidance conflicts with the repo's 5V leader supply recommendation.</v>
       </c>
     </row>
     <row r="9">
@@ -580,7 +635,7 @@
         <v>199.77</v>
       </c>
       <c r="H9" t="str">
-        <v>Buy 3 packs to get the 6x 12V follower servos required for the shared 12V rail.</v>
+        <v>Buy 3 packs to get the 6x 12V follower servos required for the shared 12V rail. Listing explicitly says 2 servos; accessory/cable contents are not explicit.</v>
       </c>
     </row>
     <row r="10">
@@ -607,7 +662,7 @@
         <v>20.4</v>
       </c>
       <c r="H10" t="str">
-        <v>Exact ST/SC serial bus board for the follower arm.</v>
+        <v>Exact repo board ASIN. Set jumpers to B-channel (USB) during LeRobot motor setup. Works with ST/SC serial bus servos.</v>
       </c>
     </row>
     <row r="11">
@@ -688,7 +743,7 @@
         <v>7.33</v>
       </c>
       <c r="H13" t="str">
-        <v>Arm hardware fill-in for M2x6 requirements.</v>
+        <v>Matches LeRobot's M2x6 requirement for the arms. Two-arm build needs about 47 M2x6 screws from the HF assembly steps.</v>
       </c>
     </row>
     <row r="14">
@@ -715,7 +770,7 @@
         <v>10.49</v>
       </c>
       <c r="H14" t="str">
-        <v>Arm hardware fill-in including M3x6 screws.</v>
+        <v>Current Amazon-only placeholder. Local LeRobot assembly docs call for M3x6 pan-head screws; this row is not an exact head-type match.</v>
       </c>
     </row>
     <row r="15">
@@ -796,7 +851,7 @@
         <v>66.28</v>
       </c>
       <c r="H17" t="str">
-        <v>Exact wrist camera row from the SO-101 optional camera docs. Shipping shown once on the listing page.</v>
+        <v>Exact SO-101 wrist-camera module model from the local optional arm docs. This is not the camera family used in LeKiwi's base-camera mount instructions.</v>
       </c>
     </row>
     <row r="18">
@@ -823,7 +878,7 @@
         <v>29.99</v>
       </c>
       <c r="H18" t="str">
-        <v>Overhead workspace camera.</v>
+        <v>Amazon.ca substitute. The local SO-101 overhead-webcam doc recommends ASIN B082X91MPP, but I could not recover a live CAD sell price from that listing.</v>
       </c>
     </row>
     <row r="19">
@@ -877,7 +932,7 @@
         <v>122.64</v>
       </c>
       <c r="H20" t="str">
-        <v>Amazon-only 100mm omni wheel option for LeKiwi. Not the VEX wheel from the original LeKiwi BOM.</v>
+        <v>Amazon-only substitute. LeKiwi's BOM references a VEX 4-inch omni wheel, not this exact Amazon.ca wheel.</v>
       </c>
     </row>
     <row r="21">
@@ -904,7 +959,7 @@
         <v>66.59</v>
       </c>
       <c r="H21" t="str">
-        <v>One 2-pack for two of the three LeKiwi base drive servos.</v>
+        <v>One 2-pack for two of the three LeKiwi base drive servos. Listing explicitly says 2 servos; accessory/cable contents are not explicit.</v>
       </c>
     </row>
     <row r="22">
@@ -931,7 +986,7 @@
         <v>45.97</v>
       </c>
       <c r="H22" t="str">
-        <v>Single 12V STS3215 to complete the 3-servo LeKiwi base drive set.</v>
+        <v>Single 12V STS3215 to complete the 3-servo LeKiwi base drive set. Listing explicitly says 1 servo; accessory/cable contents are not explicit.</v>
       </c>
     </row>
     <row r="23">
@@ -1120,7 +1175,7 @@
         <v>28.99</v>
       </c>
       <c r="H29" t="str">
-        <v>Base hardware assortment covering M2/M3/M4 needs.</v>
+        <v>Cheaper Amazon.ca substitute for LeKiwi's assorted base screw row. Covers many base machine-screw sizes, but not the arm's exact M2.5 board-mount hardware.</v>
       </c>
     </row>
     <row r="30">
@@ -1208,27 +1263,81 @@
       <c r="A33" t="str">
         <v>TOTAL: Highest Items (CAD)</v>
       </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
       <c r="G33">
         <f>SUM(G5:G32)</f>
-        <v>1288.43</v>
+        <v>1270.9</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
         <v>HST 13% (CAD)</v>
       </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
       <c r="G34">
         <f>ROUND(G33*0.13,2)</f>
-        <v>167.5</v>
+        <v>165.22</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
         <v>GRAND TOTAL (CAD)</v>
       </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
       <c r="G35">
         <f>G33+G34</f>
-        <v>1455.93</v>
+        <v>1436.12</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>